<commit_message>
Adicionado arquivos para exercícios no Power BI
</commit_message>
<xml_diff>
--- a/Power BI/aula-etl-1/1.0-4/powerbi_1.0-4_vendas_tratamento.xlsx
+++ b/Power BI/aula-etl-1/1.0-4/powerbi_1.0-4_vendas_tratamento.xlsx
@@ -17,7 +17,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+  <si>
+    <t xml:space="preserve">Relatório gerado automaticamente dia 17 de março de 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIRETORIA CENTRAL: SP</t>
+  </si>
   <si>
     <t>Vendas</t>
   </si>
@@ -34,6 +40,9 @@
     <t>Filial/Gerente</t>
   </si>
   <si>
+    <t xml:space="preserve">Diretor Regional</t>
+  </si>
+  <si>
     <t>Carlos</t>
   </si>
   <si>
@@ -43,6 +52,9 @@
     <t xml:space="preserve">RS/Marco Aurélio</t>
   </si>
   <si>
+    <t xml:space="preserve">ARAÚJO, Cristiano</t>
+  </si>
+  <si>
     <t>Max</t>
   </si>
   <si>
@@ -52,6 +64,9 @@
     <t xml:space="preserve">AC/Jonas Antunes</t>
   </si>
   <si>
+    <t xml:space="preserve">SOUZA, Aline</t>
+  </si>
+  <si>
     <t>Gabriel</t>
   </si>
   <si>
@@ -61,6 +76,9 @@
     <t xml:space="preserve">SP/Martha Maria</t>
   </si>
   <si>
+    <t xml:space="preserve">CRUZ, Penelope</t>
+  </si>
+  <si>
     <t>Fernando</t>
   </si>
   <si>
@@ -70,6 +88,9 @@
     <t xml:space="preserve">BH/Aline Santos</t>
   </si>
   <si>
+    <t xml:space="preserve">BATISTA, Anderson</t>
+  </si>
+  <si>
     <t>Charles</t>
   </si>
   <si>
@@ -79,6 +100,9 @@
     <t xml:space="preserve">RJ/Felipe Matos</t>
   </si>
   <si>
+    <t xml:space="preserve">ARAÚJO, André</t>
+  </si>
+  <si>
     <t>José</t>
   </si>
   <si>
@@ -88,6 +112,9 @@
     <t xml:space="preserve">SC/Cristiano Ruas</t>
   </si>
   <si>
+    <t xml:space="preserve">OLIVEIRA, Paulo</t>
+  </si>
+  <si>
     <t>Pedro</t>
   </si>
   <si>
@@ -95,6 +122,9 @@
   </si>
   <si>
     <t xml:space="preserve">AM/Fernando Torres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MATO, Matias</t>
   </si>
 </sst>
 </file>
@@ -608,98 +638,93 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75"/>
   <cols>
     <col bestFit="1" min="3" max="3" width="18.57421875"/>
+    <col bestFit="1" min="5" max="5" width="17.7109375"/>
   </cols>
   <sheetData>
-    <row r="1" ht="12.800000000000001">
+    <row r="1" ht="12.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+    </row>
+    <row r="2" ht="12.75">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="3" ht="12.800000000000001">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="C3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" ht="12.800000000000001">
-      <c r="A2">
+      <c r="D3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" ht="12.800000000000001">
+      <c r="A4">
         <v>88543</v>
       </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" ht="12.800000000000001">
-      <c r="A3">
-        <v>101320</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E4" t="s">
         <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5" ht="12.800000000000001">
       <c r="A5">
-        <v>89045</v>
+        <v>101320</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" ht="12.800000000000001">
-      <c r="A6">
-        <v>34579</v>
-      </c>
-      <c r="B6" t="s">
         <v>14</v>
       </c>
-      <c r="C6" t="s">
+      <c r="F5" t="s">
         <v>15</v>
-      </c>
-      <c r="E6" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="7" ht="12.800000000000001">
       <c r="A7">
-        <v>7789</v>
+        <v>89045</v>
       </c>
       <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s">
         <v>17</v>
       </c>
-      <c r="C7" t="s">
+      <c r="E7" t="s">
         <v>18</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="8" ht="12.800000000000001">
       <c r="A8">
-        <v>45678</v>
+        <v>34579</v>
       </c>
       <c r="B8" t="s">
         <v>20</v>
@@ -710,19 +735,59 @@
       <c r="E8" t="s">
         <v>22</v>
       </c>
+      <c r="F8" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="9" ht="12.800000000000001">
       <c r="A9">
+        <v>7789</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" ht="12.800000000000001">
+      <c r="A10">
+        <v>45678</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" ht="12.800000000000001">
+      <c r="A11">
         <v>33909</v>
       </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" t="s">
-        <v>25</v>
+      <c r="B11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>